<commit_message>
Diagnostico da Comunidade updated
</commit_message>
<xml_diff>
--- a/area_fernanda.xlsx
+++ b/area_fernanda.xlsx
@@ -8,19 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4d9c7f5cb995c5f2/Documentos/ProjetoPython/AfirmaSUS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F8944502-3931-4329-9712-8997F6410253}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="8_{F8944502-3931-4329-9712-8997F6410253}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E4740B6A-FDE4-478C-9B2B-07B53E33A83D}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{70F7AD8C-F2A7-4863-AAFF-90924E747BB9}"/>
   </bookViews>
   <sheets>
     <sheet name="area_fernanda" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="83">
   <si>
     <t>Carimbo de data/hora</t>
   </si>
@@ -28,39 +41,15 @@
     <t>Nome</t>
   </si>
   <si>
-    <t>Nome da rua</t>
-  </si>
-  <si>
-    <t>Numero da casa</t>
-  </si>
-  <si>
-    <t>Melhor dia na semana</t>
-  </si>
-  <si>
     <t>Turno</t>
   </si>
   <si>
-    <t>Horario</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sem horario </t>
-  </si>
-  <si>
-    <t>Pauta do encontro</t>
-  </si>
-  <si>
     <t>Solange</t>
   </si>
   <si>
     <t>RUA VILA BOM SUCESSO</t>
   </si>
   <si>
-    <t xml:space="preserve">Sem nÃºmero </t>
-  </si>
-  <si>
-    <t>SEGUNDA</t>
-  </si>
-  <si>
     <t>Manhã</t>
   </si>
   <si>
@@ -70,9 +59,6 @@
     <t xml:space="preserve">Lucicleide </t>
   </si>
   <si>
-    <t>TERÃ‡A</t>
-  </si>
-  <si>
     <t>Saneamento Básico</t>
   </si>
   <si>
@@ -88,9 +74,6 @@
     <t>RIO SAO FRANCISCO</t>
   </si>
   <si>
-    <t>SEGUNDA, TERÃ‡A, QUARTA, QUINTA, SEXTA</t>
-  </si>
-  <si>
     <t>Adriana</t>
   </si>
   <si>
@@ -103,12 +86,6 @@
     <t xml:space="preserve">MaurÃ­cio dos Santos </t>
   </si>
   <si>
-    <t>Vila da Saudade</t>
-  </si>
-  <si>
-    <t>DOMINGO</t>
-  </si>
-  <si>
     <t xml:space="preserve">Saúde do Homem </t>
   </si>
   <si>
@@ -118,9 +95,6 @@
     <t>RUA ARQUIVISTA JONATHAS CARECAS</t>
   </si>
   <si>
-    <t>SABADO</t>
-  </si>
-  <si>
     <t xml:space="preserve">Saúde da Mulher </t>
   </si>
   <si>
@@ -136,9 +110,6 @@
     <t>Cassandra</t>
   </si>
   <si>
-    <t>QUARTA</t>
-  </si>
-  <si>
     <t>Saúde do  Idoso</t>
   </si>
   <si>
@@ -178,18 +149,9 @@
     <t xml:space="preserve">Daniel Alves Nascimento </t>
   </si>
   <si>
-    <t>TERÃ‡A, QUINTA</t>
-  </si>
-  <si>
     <t>Raiane Pereira da Silva</t>
   </si>
   <si>
-    <t>S/N</t>
-  </si>
-  <si>
-    <t>DOMINGO, SEGUNDA, TERÃ‡A, QUARTA, QUINTA, SEXTA, SABADO</t>
-  </si>
-  <si>
     <t>Coleta de Lixo</t>
   </si>
   <si>
@@ -205,24 +167,15 @@
     <t xml:space="preserve">Dayana </t>
   </si>
   <si>
-    <t>Qualquer horario</t>
-  </si>
-  <si>
     <t>Hosana</t>
   </si>
   <si>
-    <t>QUINTA</t>
-  </si>
-  <si>
     <t>Diabetes</t>
   </si>
   <si>
     <t xml:space="preserve">Maria </t>
   </si>
   <si>
-    <t>SEGUNDA, QUINTA</t>
-  </si>
-  <si>
     <t>Não Especificado</t>
   </si>
   <si>
@@ -250,9 +203,6 @@
     <t>Beto</t>
   </si>
   <si>
-    <t>SEXTA</t>
-  </si>
-  <si>
     <t>Hipertensão</t>
   </si>
   <si>
@@ -293,6 +243,45 @@
   </si>
   <si>
     <t>Alexandro Pereira</t>
+  </si>
+  <si>
+    <t>Rua</t>
+  </si>
+  <si>
+    <t>Dia</t>
+  </si>
+  <si>
+    <t>Horário</t>
+  </si>
+  <si>
+    <t>Tópico</t>
+  </si>
+  <si>
+    <t>Segunda</t>
+  </si>
+  <si>
+    <t>Quarta</t>
+  </si>
+  <si>
+    <t>Quinta</t>
+  </si>
+  <si>
+    <t>Sexta</t>
+  </si>
+  <si>
+    <t>Terça</t>
+  </si>
+  <si>
+    <t>Domingo</t>
+  </si>
+  <si>
+    <t>Sábado</t>
+  </si>
+  <si>
+    <t>Qualquer Dia</t>
+  </si>
+  <si>
+    <t>NENHUM</t>
   </si>
 </sst>
 </file>
@@ -1155,10 +1144,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D1E2BA2-DA6A-4B63-9B01-A7A815EEE08F}">
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1166,952 +1164,901 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
       <c r="F1" t="s">
-        <v>5</v>
+        <v>72</v>
       </c>
       <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>46276.353472222225</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>74</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" s="2">
+        <v>5</v>
+      </c>
+      <c r="F2" s="2">
         <v>0.375</v>
       </c>
-      <c r="I2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>46276.354861111111</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3">
-        <v>705</v>
+        <v>4</v>
+      </c>
+      <c r="D3" t="s">
+        <v>78</v>
       </c>
       <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="2">
+        <v>5</v>
+      </c>
+      <c r="F3" s="2">
         <v>0.375</v>
       </c>
-      <c r="I3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>46276.376388888886</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4">
-        <v>510</v>
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
+        <v>74</v>
       </c>
       <c r="E4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" t="s">
-        <v>19</v>
-      </c>
-      <c r="G4" s="2">
+        <v>10</v>
+      </c>
+      <c r="F4" s="2">
         <v>0.58333333333333337</v>
       </c>
-      <c r="I4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>46276.379861111112</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5">
-        <v>716</v>
+        <v>12</v>
+      </c>
+      <c r="D5" t="s">
+        <v>81</v>
       </c>
       <c r="E5" t="s">
-        <v>22</v>
-      </c>
-      <c r="F5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="2">
+        <v>5</v>
+      </c>
+      <c r="F5" s="2">
         <v>0.33333333333333331</v>
       </c>
-      <c r="I5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>46276.381944444445</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6">
-        <v>716</v>
+        <v>12</v>
+      </c>
+      <c r="D6" t="s">
+        <v>74</v>
       </c>
       <c r="E6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="2">
+        <v>5</v>
+      </c>
+      <c r="F6" s="2">
         <v>0.33333333333333331</v>
       </c>
-      <c r="I6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>46276.40347222222</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
+        <v>12</v>
+      </c>
+      <c r="D7" t="s">
+        <v>74</v>
       </c>
       <c r="E7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="2">
+        <v>5</v>
+      </c>
+      <c r="F7" s="2">
         <v>0.33333333333333331</v>
       </c>
-      <c r="I7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>46276.588888888888</v>
       </c>
       <c r="B8" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>27</v>
+        <v>36</v>
+      </c>
+      <c r="D8" t="s">
+        <v>79</v>
       </c>
       <c r="E8" t="s">
-        <v>28</v>
-      </c>
-      <c r="F8" t="s">
-        <v>19</v>
-      </c>
-      <c r="G8" s="2">
+        <v>10</v>
+      </c>
+      <c r="F8" s="2">
         <v>0.54166666666666663</v>
       </c>
-      <c r="I8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>46276.592361111114</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="C9" t="s">
-        <v>31</v>
+        <v>19</v>
+      </c>
+      <c r="D9" t="s">
+        <v>80</v>
       </c>
       <c r="E9" t="s">
-        <v>32</v>
-      </c>
-      <c r="F9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9" s="2">
+        <v>5</v>
+      </c>
+      <c r="F9" s="2">
         <v>0.375</v>
       </c>
-      <c r="I9" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>46276.600694444445</v>
       </c>
       <c r="B10" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="C10" t="s">
-        <v>35</v>
-      </c>
-      <c r="I10" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+      <c r="D10" t="s">
+        <v>81</v>
+      </c>
+      <c r="G10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>46279.34652777778</v>
       </c>
       <c r="B11" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="C11" t="s">
-        <v>31</v>
-      </c>
-      <c r="D11">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="D11" t="s">
+        <v>75</v>
       </c>
       <c r="E11" t="s">
-        <v>38</v>
-      </c>
-      <c r="F11" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" s="2">
+        <v>5</v>
+      </c>
+      <c r="F11" s="2">
         <v>0.375</v>
       </c>
-      <c r="I11" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>46279.352777777778</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="C12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12">
-        <v>509</v>
+        <v>9</v>
+      </c>
+      <c r="D12" t="s">
+        <v>74</v>
       </c>
       <c r="E12" t="s">
-        <v>12</v>
-      </c>
-      <c r="F12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G12" s="2">
+        <v>5</v>
+      </c>
+      <c r="F12" s="2">
         <v>0.375</v>
       </c>
-      <c r="I12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G12" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>46279.365972222222</v>
       </c>
       <c r="B13" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="C13" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13">
-        <v>66</v>
+        <v>19</v>
+      </c>
+      <c r="D13" t="s">
+        <v>80</v>
       </c>
       <c r="E13" t="s">
-        <v>32</v>
-      </c>
-      <c r="F13" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" s="2">
+        <v>5</v>
+      </c>
+      <c r="F13" s="2">
         <v>0.375</v>
       </c>
-      <c r="I13" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G13" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>46279.414583333331</v>
       </c>
       <c r="B14" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="C14" t="s">
-        <v>31</v>
-      </c>
-      <c r="D14">
-        <v>30</v>
+        <v>19</v>
+      </c>
+      <c r="D14" t="s">
+        <v>74</v>
       </c>
       <c r="E14" t="s">
-        <v>12</v>
-      </c>
-      <c r="F14" t="s">
-        <v>19</v>
-      </c>
-      <c r="G14" s="2">
+        <v>10</v>
+      </c>
+      <c r="F14" s="2">
         <v>0.58333333333333337</v>
       </c>
-      <c r="I14" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G14" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>46280.375</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="C15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" t="s">
+        <v>78</v>
+      </c>
+      <c r="E15" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="2">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="G15" t="s">
         <v>31</v>
       </c>
-      <c r="D15">
-        <v>0</v>
-      </c>
-      <c r="E15" t="s">
-        <v>16</v>
-      </c>
-      <c r="F15" t="s">
-        <v>19</v>
-      </c>
-      <c r="G15" s="2">
-        <v>0.58333333333333337</v>
-      </c>
-      <c r="I15" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>46280.376388888886</v>
       </c>
       <c r="B16" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="C16" t="s">
-        <v>35</v>
+        <v>22</v>
+      </c>
+      <c r="D16" t="s">
+        <v>80</v>
       </c>
       <c r="E16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F16" t="s">
-        <v>13</v>
-      </c>
-      <c r="G16" s="2">
+        <v>5</v>
+      </c>
+      <c r="F16" s="2">
         <v>0.33333333333333331</v>
       </c>
-      <c r="I16" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>46280.386111111111</v>
       </c>
       <c r="B17" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="C17" t="s">
-        <v>31</v>
-      </c>
-      <c r="D17">
-        <v>117</v>
+        <v>19</v>
+      </c>
+      <c r="D17" t="s">
+        <v>81</v>
       </c>
       <c r="E17" t="s">
-        <v>22</v>
-      </c>
-      <c r="F17" t="s">
-        <v>19</v>
-      </c>
-      <c r="G17" s="2">
+        <v>10</v>
+      </c>
+      <c r="F17" s="2">
         <v>0.5625</v>
       </c>
-      <c r="I17" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>46280.386805555558</v>
       </c>
       <c r="B18" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="C18" t="s">
-        <v>50</v>
-      </c>
-      <c r="D18">
-        <v>15</v>
+        <v>36</v>
+      </c>
+      <c r="D18" t="s">
+        <v>74</v>
       </c>
       <c r="E18" t="s">
-        <v>12</v>
-      </c>
-      <c r="F18" t="s">
-        <v>19</v>
-      </c>
-      <c r="G18" s="2">
+        <v>10</v>
+      </c>
+      <c r="F18" s="2">
         <v>0.5625</v>
       </c>
-      <c r="I18" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G18" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>46287.354166666664</v>
       </c>
       <c r="B19" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="C19" t="s">
-        <v>18</v>
-      </c>
-      <c r="D19">
-        <v>514</v>
+        <v>9</v>
+      </c>
+      <c r="D19" t="s">
+        <v>78</v>
       </c>
       <c r="E19" t="s">
-        <v>52</v>
-      </c>
-      <c r="F19" t="s">
-        <v>13</v>
-      </c>
-      <c r="G19" s="2">
+        <v>5</v>
+      </c>
+      <c r="F19" s="2">
         <v>0.33333333333333331</v>
       </c>
-      <c r="I19" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G19" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>46287.356249999997</v>
       </c>
       <c r="B20" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="C20" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="D20" t="s">
-        <v>54</v>
+        <v>81</v>
       </c>
       <c r="E20" t="s">
-        <v>55</v>
-      </c>
-      <c r="F20" t="s">
-        <v>19</v>
-      </c>
-      <c r="G20" s="2">
+        <v>10</v>
+      </c>
+      <c r="F20" s="2">
         <v>0.54166666666666663</v>
       </c>
-      <c r="I20" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G20" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>46287.400694444441</v>
       </c>
       <c r="B21" t="s">
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="C21" t="s">
-        <v>18</v>
-      </c>
-      <c r="D21">
-        <v>519</v>
+        <v>9</v>
+      </c>
+      <c r="D21" t="s">
+        <v>81</v>
       </c>
       <c r="E21" t="s">
-        <v>55</v>
-      </c>
-      <c r="F21" t="s">
-        <v>19</v>
-      </c>
-      <c r="G21" s="2">
+        <v>10</v>
+      </c>
+      <c r="F21" s="2">
         <v>0.66666666666666663</v>
       </c>
-      <c r="I21" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G21" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>46287.401388888888</v>
       </c>
       <c r="B22" t="s">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="C22" t="s">
-        <v>50</v>
+        <v>36</v>
+      </c>
+      <c r="D22" t="s">
+        <v>78</v>
       </c>
       <c r="E22" t="s">
-        <v>16</v>
-      </c>
-      <c r="F22" t="s">
-        <v>59</v>
-      </c>
-      <c r="G22" s="2">
+        <v>42</v>
+      </c>
+      <c r="F22" s="2">
         <v>0.58333333333333337</v>
       </c>
-      <c r="I22" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G22" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>46287.404166666667</v>
       </c>
       <c r="B23" t="s">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="C23" t="s">
-        <v>21</v>
+        <v>12</v>
+      </c>
+      <c r="D23" t="s">
+        <v>74</v>
       </c>
       <c r="E23" t="s">
-        <v>12</v>
-      </c>
-      <c r="F23" t="s">
-        <v>13</v>
-      </c>
-      <c r="G23" s="2">
+        <v>5</v>
+      </c>
+      <c r="F23" s="2">
         <v>0.58333333333333337</v>
       </c>
-      <c r="H23" t="s">
-        <v>61</v>
-      </c>
-      <c r="I23" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G23" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>46287.404861111114</v>
       </c>
       <c r="B24" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="C24" t="s">
-        <v>21</v>
+        <v>12</v>
+      </c>
+      <c r="D24" t="s">
+        <v>76</v>
       </c>
       <c r="E24" t="s">
-        <v>63</v>
-      </c>
-      <c r="F24" t="s">
-        <v>19</v>
-      </c>
-      <c r="G24" s="2">
+        <v>10</v>
+      </c>
+      <c r="F24" s="2">
         <v>0.625</v>
       </c>
-      <c r="I24" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>46287.40625</v>
       </c>
       <c r="B25" t="s">
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="C25" t="s">
-        <v>21</v>
+        <v>12</v>
+      </c>
+      <c r="D25" t="s">
+        <v>76</v>
       </c>
       <c r="E25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F25" t="s">
-        <v>13</v>
-      </c>
-      <c r="G25" s="2">
+        <v>5</v>
+      </c>
+      <c r="F25" s="2">
         <v>0.33333333333333331</v>
       </c>
-      <c r="I25" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G25" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>46287.406944444447</v>
       </c>
       <c r="B26" t="s">
-        <v>68</v>
+        <v>48</v>
       </c>
       <c r="C26" t="s">
-        <v>21</v>
-      </c>
-      <c r="D26">
-        <v>710</v>
+        <v>12</v>
+      </c>
+      <c r="D26" t="s">
+        <v>80</v>
       </c>
       <c r="E26" t="s">
-        <v>32</v>
-      </c>
-      <c r="F26" t="s">
-        <v>19</v>
-      </c>
-      <c r="G26" s="2">
+        <v>10</v>
+      </c>
+      <c r="F26" s="2">
         <v>0.625</v>
       </c>
-      <c r="I26" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G26" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>46287.408333333333</v>
       </c>
       <c r="B27" t="s">
-        <v>69</v>
+        <v>49</v>
       </c>
       <c r="C27" t="s">
-        <v>21</v>
+        <v>12</v>
+      </c>
+      <c r="D27" t="s">
+        <v>81</v>
       </c>
       <c r="E27" t="s">
-        <v>55</v>
-      </c>
-      <c r="F27" t="s">
-        <v>19</v>
-      </c>
-      <c r="G27" s="2">
+        <v>10</v>
+      </c>
+      <c r="F27" s="2">
         <v>0.54166666666666663</v>
       </c>
-      <c r="I27" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G27" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>46287.408333333333</v>
       </c>
       <c r="B28" t="s">
-        <v>71</v>
+        <v>51</v>
       </c>
       <c r="C28" t="s">
-        <v>21</v>
+        <v>12</v>
+      </c>
+      <c r="D28" t="s">
+        <v>75</v>
       </c>
       <c r="E28" t="s">
-        <v>38</v>
-      </c>
-      <c r="F28" t="s">
-        <v>13</v>
-      </c>
-      <c r="G28" s="2">
+        <v>5</v>
+      </c>
+      <c r="F28" s="2">
         <v>0.41666666666666669</v>
       </c>
-      <c r="I28" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G28" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>46287.413194444445</v>
       </c>
       <c r="B29" t="s">
-        <v>73</v>
+        <v>53</v>
       </c>
       <c r="C29" t="s">
-        <v>35</v>
-      </c>
-      <c r="F29" t="s">
-        <v>13</v>
-      </c>
-      <c r="G29" s="2">
+        <v>22</v>
+      </c>
+      <c r="D29" t="s">
+        <v>81</v>
+      </c>
+      <c r="E29" t="s">
+        <v>5</v>
+      </c>
+      <c r="F29" s="2">
         <v>0.29166666666666669</v>
       </c>
-      <c r="I29" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G29" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>46287.415277777778</v>
       </c>
       <c r="B30" t="s">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="C30" t="s">
-        <v>35</v>
-      </c>
-      <c r="D30">
-        <v>610</v>
+        <v>22</v>
+      </c>
+      <c r="D30" t="s">
+        <v>80</v>
       </c>
       <c r="E30" t="s">
-        <v>32</v>
-      </c>
-      <c r="F30" t="s">
-        <v>19</v>
-      </c>
-      <c r="G30" s="2">
+        <v>10</v>
+      </c>
+      <c r="F30" s="2">
         <v>0.58333333333333337</v>
       </c>
-      <c r="I30" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G30" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>46287.416666666664</v>
       </c>
       <c r="B31" t="s">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="C31" t="s">
-        <v>35</v>
+        <v>22</v>
+      </c>
+      <c r="D31" t="s">
+        <v>77</v>
       </c>
       <c r="E31" t="s">
-        <v>76</v>
-      </c>
-      <c r="F31" t="s">
-        <v>19</v>
-      </c>
-      <c r="G31" s="2">
+        <v>10</v>
+      </c>
+      <c r="F31" s="2">
         <v>0.625</v>
       </c>
-      <c r="I31" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G31" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>46287.419444444444</v>
       </c>
       <c r="B32" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="C32" t="s">
-        <v>35</v>
-      </c>
-      <c r="I32" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+      <c r="D32" t="s">
+        <v>81</v>
+      </c>
+      <c r="G32" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>46287.424305555556</v>
       </c>
       <c r="B33" t="s">
-        <v>79</v>
+        <v>58</v>
       </c>
       <c r="C33" t="s">
-        <v>35</v>
+        <v>22</v>
+      </c>
+      <c r="D33" t="s">
+        <v>78</v>
       </c>
       <c r="E33" t="s">
-        <v>16</v>
-      </c>
-      <c r="F33" t="s">
-        <v>13</v>
-      </c>
-      <c r="G33" s="2">
+        <v>5</v>
+      </c>
+      <c r="F33" s="2">
         <v>0.41666666666666669</v>
       </c>
-      <c r="I33" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G33" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>46287.427083333336</v>
       </c>
       <c r="B34" t="s">
-        <v>80</v>
+        <v>59</v>
       </c>
       <c r="C34" t="s">
-        <v>31</v>
+        <v>19</v>
+      </c>
+      <c r="D34" t="s">
+        <v>76</v>
       </c>
       <c r="E34" t="s">
-        <v>63</v>
-      </c>
-      <c r="F34" t="s">
-        <v>13</v>
-      </c>
-      <c r="G34" s="2">
+        <v>5</v>
+      </c>
+      <c r="F34" s="2">
         <v>0.33333333333333331</v>
       </c>
-      <c r="I34" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G34" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
         <v>46287.427083333336</v>
       </c>
       <c r="B35" t="s">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="C35" t="s">
-        <v>18</v>
+        <v>9</v>
+      </c>
+      <c r="D35" t="s">
+        <v>74</v>
       </c>
       <c r="E35" t="s">
-        <v>12</v>
-      </c>
-      <c r="F35" t="s">
-        <v>13</v>
-      </c>
-      <c r="G35" s="2">
+        <v>5</v>
+      </c>
+      <c r="F35" s="2">
         <v>0.375</v>
       </c>
-      <c r="I35" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G35" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
         <v>46287.429861111108</v>
       </c>
       <c r="B36" t="s">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="C36" t="s">
-        <v>31</v>
+        <v>19</v>
+      </c>
+      <c r="D36" t="s">
+        <v>76</v>
       </c>
       <c r="E36" t="s">
-        <v>63</v>
-      </c>
-      <c r="F36" t="s">
-        <v>13</v>
-      </c>
-      <c r="G36" s="2">
+        <v>5</v>
+      </c>
+      <c r="F36" s="2">
         <v>0.33333333333333331</v>
       </c>
-      <c r="I36" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G36" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
         <v>46287.430555555555</v>
       </c>
       <c r="B37" t="s">
-        <v>84</v>
+        <v>63</v>
       </c>
       <c r="C37" t="s">
-        <v>31</v>
+        <v>19</v>
+      </c>
+      <c r="D37" t="s">
+        <v>78</v>
       </c>
       <c r="E37" t="s">
-        <v>16</v>
-      </c>
-      <c r="F37" t="s">
-        <v>13</v>
-      </c>
-      <c r="G37" s="2">
+        <v>5</v>
+      </c>
+      <c r="F37" s="2">
         <v>0.41666666666666669</v>
       </c>
-      <c r="I37" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G37" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
         <v>46287.436111111114</v>
       </c>
       <c r="B38" t="s">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="C38" t="s">
-        <v>35</v>
+        <v>22</v>
+      </c>
+      <c r="D38" t="s">
+        <v>78</v>
       </c>
       <c r="E38" t="s">
-        <v>16</v>
-      </c>
-      <c r="F38" t="s">
-        <v>13</v>
-      </c>
-      <c r="G38" s="2">
+        <v>5</v>
+      </c>
+      <c r="F38" s="2">
         <v>0.375</v>
       </c>
-      <c r="I38" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G38" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
         <v>46287.438194444447</v>
       </c>
       <c r="B39" t="s">
-        <v>88</v>
+        <v>67</v>
+      </c>
+      <c r="C39" t="s">
+        <v>82</v>
+      </c>
+      <c r="D39" t="s">
+        <v>76</v>
       </c>
       <c r="E39" t="s">
-        <v>63</v>
-      </c>
-      <c r="F39" t="s">
-        <v>19</v>
-      </c>
-      <c r="G39" s="2">
+        <v>10</v>
+      </c>
+      <c r="F39" s="2">
         <v>0.54166666666666663</v>
       </c>
-      <c r="I39" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G39" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
         <v>46290.375694444447</v>
       </c>
       <c r="B40" t="s">
-        <v>90</v>
+        <v>69</v>
       </c>
       <c r="C40" t="s">
+        <v>4</v>
+      </c>
+      <c r="D40" t="s">
+        <v>77</v>
+      </c>
+      <c r="E40" t="s">
         <v>10</v>
       </c>
-      <c r="D40">
-        <v>722</v>
-      </c>
-      <c r="E40" t="s">
-        <v>76</v>
-      </c>
-      <c r="F40" t="s">
-        <v>19</v>
-      </c>
-      <c r="G40" s="2">
+      <c r="F40" s="2">
         <v>0.58333333333333337</v>
       </c>
-      <c r="I40" t="s">
-        <v>17</v>
+      <c r="G40" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>